<commit_message>
model and excel files updated
</commit_message>
<xml_diff>
--- a/IA_CCBS_BANK_SIDE/AccountOther/LoanAccountOpening_InstantProcess.xlsx
+++ b/IA_CCBS_BANK_SIDE/AccountOther/LoanAccountOpening_InstantProcess.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Sw\Relational_Files\iApply\Interfaces\Interfaces_plus_allbanks\IA_CCBS_BANK_SIDE\AccountOther\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kmilos\source\repos\iApply_CCBS_API\IA_CCBS_BANK_SIDE\AccountOther\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E31733D-87A5-434A-9D65-671FA85B02E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4234C863-96FE-4972-B220-969F8E23A493}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-5550" windowWidth="30960" windowHeight="16920" xr2:uid="{68F28061-2ECD-4B0A-AB1D-3A449686159F}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{68F28061-2ECD-4B0A-AB1D-3A449686159F}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="3" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="112">
   <si>
     <t>Description</t>
   </si>
@@ -352,6 +352,21 @@
   </si>
   <si>
     <t>iban_account_cd</t>
+  </si>
+  <si>
+    <t>MarginFixedIR</t>
+  </si>
+  <si>
+    <t>MarginFloatingIR</t>
+  </si>
+  <si>
+    <t>FloatingLocal</t>
+  </si>
+  <si>
+    <t>decimal (19,2)</t>
+  </si>
+  <si>
+    <t>string</t>
   </si>
 </sst>
 </file>
@@ -520,7 +535,7 @@
     <xf numFmtId="0" fontId="12" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="12" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -599,6 +614,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="20% - Accent4" xfId="1" builtinId="42"/>
@@ -1026,7 +1042,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{A6ACF92C-1104-4C93-8F8B-A938A4312D3B}" name="Table2" displayName="Table2" ref="B2:G31" totalsRowShown="0" headerRowDxfId="21" dataDxfId="20" headerRowCellStyle="Normal" dataCellStyle="Normal">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{A6ACF92C-1104-4C93-8F8B-A938A4312D3B}" name="Table2" displayName="Table2" ref="B2:G34" totalsRowShown="0" headerRowDxfId="21" dataDxfId="20" headerRowCellStyle="Normal" dataCellStyle="Normal">
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:G31">
     <sortCondition ref="B3"/>
   </sortState>
@@ -1355,20 +1371,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3BB8ACDA-C8F4-4728-9499-8B46BAA74AEA}">
   <dimension ref="B2:C14"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="4.5703125" customWidth="1"/>
-    <col min="2" max="2" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="41.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="4.5546875" customWidth="1"/>
+    <col min="2" max="2" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="41.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:3" ht="31.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:3" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="17"/>
       <c r="C2" s="18" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B3" s="18" t="s">
         <v>10</v>
       </c>
@@ -1376,7 +1392,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B4" s="18" t="s">
         <v>12</v>
       </c>
@@ -1384,7 +1400,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="5" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B5" s="18" t="s">
         <v>13</v>
       </c>
@@ -1392,7 +1408,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B6" s="21" t="s">
         <v>21</v>
       </c>
@@ -1400,7 +1416,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="7" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B7" s="18" t="s">
         <v>15</v>
       </c>
@@ -1408,11 +1424,11 @@
         <v>16</v>
       </c>
     </row>
-    <row r="8" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B8" s="18"/>
       <c r="C8" s="19"/>
     </row>
-    <row r="9" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B9" s="18" t="s">
         <v>17</v>
       </c>
@@ -1420,7 +1436,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="10" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B10" s="18" t="s">
         <v>19</v>
       </c>
@@ -1428,15 +1444,15 @@
         <v>29</v>
       </c>
     </row>
-    <row r="11" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B11" s="18"/>
       <c r="C11" s="19"/>
     </row>
-    <row r="12" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B12" s="18"/>
       <c r="C12" s="19"/>
     </row>
-    <row r="13" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B13" s="18" t="s">
         <v>20</v>
       </c>
@@ -1444,7 +1460,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="14" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B14" s="18"/>
       <c r="C14" s="19"/>
     </row>
@@ -1456,20 +1472,20 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{03AC1DB5-1548-45C4-B0E5-7097191C5328}">
   <dimension ref="B1:G105"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="16.5" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="1.42578125" style="2" customWidth="1"/>
-    <col min="2" max="2" width="6.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="27.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="30.85546875" style="2" customWidth="1"/>
-    <col min="6" max="6" width="19.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.85546875" style="2" customWidth="1"/>
-    <col min="8" max="16384" width="9.140625" style="2"/>
+    <col min="1" max="1" width="1.44140625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="6.5546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27.5546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.33203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="30.88671875" style="2" customWidth="1"/>
+    <col min="6" max="6" width="19.6640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.88671875" style="2" customWidth="1"/>
+    <col min="8" max="16384" width="9.109375" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:7" ht="8.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="2" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:7" ht="8.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="22" t="s">
         <v>8</v>
       </c>
@@ -1489,7 +1505,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="2:7" s="1" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:7" s="1" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B3">
         <v>1</v>
       </c>
@@ -1507,7 +1523,7 @@
       </c>
       <c r="G3" s="26"/>
     </row>
-    <row r="4" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4">
         <v>2</v>
       </c>
@@ -1525,7 +1541,7 @@
       </c>
       <c r="G4" s="26"/>
     </row>
-    <row r="5" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5">
         <v>3</v>
       </c>
@@ -1543,7 +1559,7 @@
       </c>
       <c r="G5" s="26"/>
     </row>
-    <row r="6" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6">
         <v>4</v>
       </c>
@@ -1561,7 +1577,7 @@
       </c>
       <c r="G6" s="26"/>
     </row>
-    <row r="7" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7">
         <v>5</v>
       </c>
@@ -1579,7 +1595,7 @@
       </c>
       <c r="G7" s="26"/>
     </row>
-    <row r="8" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B8">
         <v>6</v>
       </c>
@@ -1597,7 +1613,7 @@
       </c>
       <c r="G8" s="27"/>
     </row>
-    <row r="9" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9">
         <v>7</v>
       </c>
@@ -1615,7 +1631,7 @@
       </c>
       <c r="G9" s="26"/>
     </row>
-    <row r="10" spans="2:7" s="4" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:7" s="4" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10">
         <v>8</v>
       </c>
@@ -1633,7 +1649,7 @@
       </c>
       <c r="G10" s="27"/>
     </row>
-    <row r="11" spans="2:7" s="4" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:7" s="4" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11">
         <v>9</v>
       </c>
@@ -1651,7 +1667,7 @@
       </c>
       <c r="G11" s="26"/>
     </row>
-    <row r="12" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12">
         <v>10</v>
       </c>
@@ -1669,7 +1685,7 @@
       </c>
       <c r="G12" s="26"/>
     </row>
-    <row r="13" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B13">
         <v>11</v>
       </c>
@@ -1687,7 +1703,7 @@
       </c>
       <c r="G13" s="26"/>
     </row>
-    <row r="14" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B14">
         <v>12</v>
       </c>
@@ -1705,7 +1721,7 @@
       </c>
       <c r="G14" s="26"/>
     </row>
-    <row r="15" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B15">
         <v>13</v>
       </c>
@@ -1723,7 +1739,7 @@
       </c>
       <c r="G15" s="26"/>
     </row>
-    <row r="16" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16">
         <v>14</v>
       </c>
@@ -1741,7 +1757,7 @@
       </c>
       <c r="G16" s="26"/>
     </row>
-    <row r="17" spans="2:7" s="1" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:7" s="1" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B17">
         <v>15</v>
       </c>
@@ -1759,7 +1775,7 @@
       </c>
       <c r="G17" s="26"/>
     </row>
-    <row r="18" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B18">
         <v>16</v>
       </c>
@@ -1777,7 +1793,7 @@
       </c>
       <c r="G18" s="26"/>
     </row>
-    <row r="19" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B19">
         <v>17</v>
       </c>
@@ -1795,7 +1811,7 @@
       </c>
       <c r="G19" s="26"/>
     </row>
-    <row r="20" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B20">
         <v>18</v>
       </c>
@@ -1813,7 +1829,7 @@
       </c>
       <c r="G20" s="26"/>
     </row>
-    <row r="21" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B21">
         <v>19</v>
       </c>
@@ -1831,7 +1847,7 @@
       </c>
       <c r="G21" s="26"/>
     </row>
-    <row r="22" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B22">
         <v>20</v>
       </c>
@@ -1849,7 +1865,7 @@
       </c>
       <c r="G22" s="26"/>
     </row>
-    <row r="23" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B23">
         <v>21</v>
       </c>
@@ -1867,7 +1883,7 @@
       </c>
       <c r="G23" s="26"/>
     </row>
-    <row r="24" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B24">
         <v>22</v>
       </c>
@@ -1885,7 +1901,7 @@
       </c>
       <c r="G24" s="26"/>
     </row>
-    <row r="25" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B25">
         <v>23</v>
       </c>
@@ -1903,7 +1919,7 @@
       </c>
       <c r="G25" s="26"/>
     </row>
-    <row r="26" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B26">
         <v>24</v>
       </c>
@@ -1921,7 +1937,7 @@
       </c>
       <c r="G26" s="26"/>
     </row>
-    <row r="27" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B27">
         <v>25</v>
       </c>
@@ -1939,7 +1955,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B28">
         <v>26</v>
       </c>
@@ -1957,7 +1973,7 @@
       </c>
       <c r="G28" s="27"/>
     </row>
-    <row r="29" spans="2:7" s="4" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:7" s="4" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B29">
         <v>27</v>
       </c>
@@ -1975,7 +1991,7 @@
       </c>
       <c r="G29" s="26"/>
     </row>
-    <row r="30" spans="2:7" s="4" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:7" s="4" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B30">
         <v>28</v>
       </c>
@@ -1993,7 +2009,7 @@
       </c>
       <c r="G30" s="26"/>
     </row>
-    <row r="31" spans="2:7" s="4" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:7" s="4" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B31">
         <v>29</v>
       </c>
@@ -2011,29 +2027,61 @@
       </c>
       <c r="G31" s="26"/>
     </row>
-    <row r="32" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B32" s="3"/>
-      <c r="C32" s="3"/>
-      <c r="D32" s="5"/>
-      <c r="E32" s="5"/>
-      <c r="F32" s="5"/>
-      <c r="G32" s="6"/>
-    </row>
-    <row r="33" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D33" s="5"/>
-      <c r="E33" s="5"/>
-      <c r="F33" s="5"/>
-      <c r="G33" s="6"/>
-    </row>
-    <row r="34" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B34" s="1"/>
-      <c r="C34" s="1"/>
-      <c r="D34" s="7"/>
-      <c r="E34" s="7"/>
-      <c r="F34" s="7"/>
-      <c r="G34" s="8"/>
-    </row>
-    <row r="35" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B32">
+        <v>30</v>
+      </c>
+      <c r="C32" s="28" t="s">
+        <v>107</v>
+      </c>
+      <c r="D32" s="28" t="s">
+        <v>107</v>
+      </c>
+      <c r="E32" s="26" t="s">
+        <v>110</v>
+      </c>
+      <c r="F32" s="26" t="s">
+        <v>32</v>
+      </c>
+      <c r="G32" s="28"/>
+    </row>
+    <row r="33" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B33">
+        <v>31</v>
+      </c>
+      <c r="C33" s="28" t="s">
+        <v>108</v>
+      </c>
+      <c r="D33" s="28" t="s">
+        <v>108</v>
+      </c>
+      <c r="E33" s="26" t="s">
+        <v>110</v>
+      </c>
+      <c r="F33" s="26" t="s">
+        <v>32</v>
+      </c>
+      <c r="G33" s="28"/>
+    </row>
+    <row r="34" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B34">
+        <v>32</v>
+      </c>
+      <c r="C34" s="28" t="s">
+        <v>109</v>
+      </c>
+      <c r="D34" s="28" t="s">
+        <v>109</v>
+      </c>
+      <c r="E34" s="28" t="s">
+        <v>111</v>
+      </c>
+      <c r="F34" s="26" t="s">
+        <v>32</v>
+      </c>
+      <c r="G34" s="28"/>
+    </row>
+    <row r="35" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B35" s="2"/>
       <c r="C35" s="2"/>
       <c r="D35" s="5"/>
@@ -2041,7 +2089,7 @@
       <c r="F35" s="5"/>
       <c r="G35" s="6"/>
     </row>
-    <row r="36" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B36" s="2"/>
       <c r="C36" s="2"/>
       <c r="D36" s="5"/>
@@ -2049,25 +2097,25 @@
       <c r="F36" s="5"/>
       <c r="G36" s="6"/>
     </row>
-    <row r="37" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D37" s="5"/>
       <c r="E37" s="5"/>
       <c r="F37" s="5"/>
       <c r="G37" s="6"/>
     </row>
-    <row r="38" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D38" s="5"/>
       <c r="E38" s="5"/>
       <c r="F38" s="5"/>
       <c r="G38" s="6"/>
     </row>
-    <row r="39" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D39" s="5"/>
       <c r="E39" s="5"/>
       <c r="F39" s="5"/>
       <c r="G39" s="6"/>
     </row>
-    <row r="40" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B40" s="3"/>
       <c r="C40" s="3"/>
       <c r="D40" s="5"/>
@@ -2075,7 +2123,7 @@
       <c r="F40" s="5"/>
       <c r="G40" s="6"/>
     </row>
-    <row r="41" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B41" s="3"/>
       <c r="C41" s="3"/>
       <c r="D41" s="7"/>
@@ -2083,7 +2131,7 @@
       <c r="F41" s="7"/>
       <c r="G41" s="8"/>
     </row>
-    <row r="42" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B42" s="3"/>
       <c r="C42" s="3"/>
       <c r="D42" s="7"/>
@@ -2091,7 +2139,7 @@
       <c r="F42" s="7"/>
       <c r="G42" s="8"/>
     </row>
-    <row r="43" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B43" s="3"/>
       <c r="C43" s="3"/>
       <c r="D43" s="5"/>
@@ -2099,7 +2147,7 @@
       <c r="F43" s="5"/>
       <c r="G43" s="6"/>
     </row>
-    <row r="44" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B44" s="3"/>
       <c r="C44" s="3"/>
       <c r="D44" s="5"/>
@@ -2107,13 +2155,13 @@
       <c r="F44" s="5"/>
       <c r="G44" s="6"/>
     </row>
-    <row r="45" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D45" s="5"/>
       <c r="E45" s="5"/>
       <c r="F45" s="5"/>
       <c r="G45" s="6"/>
     </row>
-    <row r="46" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B46" s="3"/>
       <c r="C46" s="3"/>
       <c r="D46" s="5"/>
@@ -2121,13 +2169,13 @@
       <c r="F46" s="5"/>
       <c r="G46" s="6"/>
     </row>
-    <row r="47" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D47" s="5"/>
       <c r="E47" s="5"/>
       <c r="F47" s="5"/>
       <c r="G47" s="6"/>
     </row>
-    <row r="48" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B48" s="4"/>
       <c r="C48" s="4"/>
       <c r="D48" s="9"/>
@@ -2135,7 +2183,7 @@
       <c r="F48" s="10"/>
       <c r="G48" s="9"/>
     </row>
-    <row r="49" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B49" s="4"/>
       <c r="C49" s="4"/>
       <c r="D49" s="9"/>
@@ -2143,7 +2191,7 @@
       <c r="F49" s="10"/>
       <c r="G49" s="9"/>
     </row>
-    <row r="50" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B50" s="4"/>
       <c r="C50" s="4"/>
       <c r="D50" s="9"/>
@@ -2151,7 +2199,7 @@
       <c r="F50" s="10"/>
       <c r="G50" s="9"/>
     </row>
-    <row r="51" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B51" s="4"/>
       <c r="C51" s="4"/>
       <c r="D51" s="9"/>
@@ -2159,7 +2207,7 @@
       <c r="F51" s="10"/>
       <c r="G51" s="9"/>
     </row>
-    <row r="52" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B52" s="4"/>
       <c r="C52" s="4"/>
       <c r="D52" s="9"/>
@@ -2167,7 +2215,7 @@
       <c r="F52" s="10"/>
       <c r="G52" s="9"/>
     </row>
-    <row r="53" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B53" s="4"/>
       <c r="C53" s="4"/>
       <c r="D53" s="9"/>
@@ -2175,19 +2223,19 @@
       <c r="F53" s="10"/>
       <c r="G53" s="9"/>
     </row>
-    <row r="54" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D54" s="11"/>
       <c r="E54" s="11"/>
       <c r="F54" s="11"/>
       <c r="G54" s="12"/>
     </row>
-    <row r="55" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D55" s="5"/>
       <c r="E55" s="5"/>
       <c r="F55" s="5"/>
       <c r="G55" s="6"/>
     </row>
-    <row r="56" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B56" s="3"/>
       <c r="C56" s="3"/>
       <c r="D56" s="5"/>
@@ -2195,7 +2243,7 @@
       <c r="F56" s="5"/>
       <c r="G56" s="6"/>
     </row>
-    <row r="57" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B57" s="13"/>
       <c r="C57" s="13"/>
       <c r="D57" s="11"/>
@@ -2203,7 +2251,7 @@
       <c r="F57" s="11"/>
       <c r="G57" s="12"/>
     </row>
-    <row r="58" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B58" s="4"/>
       <c r="C58" s="4"/>
       <c r="D58" s="11"/>
@@ -2211,7 +2259,7 @@
       <c r="F58" s="11"/>
       <c r="G58" s="12"/>
     </row>
-    <row r="59" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B59" s="4"/>
       <c r="C59" s="4"/>
       <c r="D59" s="11"/>
@@ -2219,7 +2267,7 @@
       <c r="F59" s="11"/>
       <c r="G59" s="12"/>
     </row>
-    <row r="60" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B60" s="4"/>
       <c r="C60" s="4"/>
       <c r="D60" s="11"/>
@@ -2227,7 +2275,7 @@
       <c r="F60" s="11"/>
       <c r="G60" s="12"/>
     </row>
-    <row r="61" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B61" s="4"/>
       <c r="C61" s="4"/>
       <c r="D61" s="14"/>
@@ -2235,13 +2283,13 @@
       <c r="F61" s="14"/>
       <c r="G61" s="15"/>
     </row>
-    <row r="62" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D62" s="5"/>
       <c r="E62" s="5"/>
       <c r="F62" s="5"/>
       <c r="G62" s="6"/>
     </row>
-    <row r="63" spans="2:7" s="16" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="2:7" s="16" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B63" s="2"/>
       <c r="C63" s="2"/>
       <c r="D63" s="5"/>
@@ -2249,19 +2297,19 @@
       <c r="F63" s="5"/>
       <c r="G63" s="6"/>
     </row>
-    <row r="64" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D64" s="5"/>
       <c r="E64" s="5"/>
       <c r="F64" s="5"/>
       <c r="G64" s="6"/>
     </row>
-    <row r="65" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D65" s="5"/>
       <c r="E65" s="5"/>
       <c r="F65" s="5"/>
       <c r="G65" s="6"/>
     </row>
-    <row r="66" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B66" s="3"/>
       <c r="C66" s="3"/>
       <c r="D66" s="5"/>
@@ -2269,7 +2317,7 @@
       <c r="F66" s="5"/>
       <c r="G66" s="6"/>
     </row>
-    <row r="67" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B67" s="3"/>
       <c r="C67" s="3"/>
       <c r="D67" s="11"/>
@@ -2277,7 +2325,7 @@
       <c r="F67" s="11"/>
       <c r="G67" s="12"/>
     </row>
-    <row r="68" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B68" s="3"/>
       <c r="C68" s="3"/>
       <c r="D68" s="11"/>
@@ -2285,49 +2333,49 @@
       <c r="F68" s="11"/>
       <c r="G68" s="12"/>
     </row>
-    <row r="69" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D69" s="5"/>
       <c r="E69" s="5"/>
       <c r="F69" s="5"/>
       <c r="G69" s="6"/>
     </row>
-    <row r="70" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D70" s="5"/>
       <c r="E70" s="5"/>
       <c r="F70" s="5"/>
       <c r="G70" s="6"/>
     </row>
-    <row r="71" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D71" s="11"/>
       <c r="E71" s="11"/>
       <c r="F71" s="11"/>
       <c r="G71" s="12"/>
     </row>
-    <row r="72" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D72" s="5"/>
       <c r="E72" s="5"/>
       <c r="F72" s="5"/>
       <c r="G72" s="6"/>
     </row>
-    <row r="73" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D73" s="5"/>
       <c r="E73" s="5"/>
       <c r="F73" s="5"/>
       <c r="G73" s="6"/>
     </row>
-    <row r="74" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D74" s="5"/>
       <c r="E74" s="5"/>
       <c r="F74" s="5"/>
       <c r="G74" s="6"/>
     </row>
-    <row r="75" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D75" s="5"/>
       <c r="E75" s="5"/>
       <c r="F75" s="5"/>
       <c r="G75" s="6"/>
     </row>
-    <row r="76" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B76" s="3"/>
       <c r="C76" s="3"/>
       <c r="D76" s="5"/>
@@ -2335,7 +2383,7 @@
       <c r="F76" s="5"/>
       <c r="G76" s="6"/>
     </row>
-    <row r="77" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B77" s="3"/>
       <c r="C77" s="3"/>
       <c r="D77" s="5"/>
@@ -2343,7 +2391,7 @@
       <c r="F77" s="5"/>
       <c r="G77" s="6"/>
     </row>
-    <row r="78" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B78" s="3"/>
       <c r="C78" s="3"/>
       <c r="D78" s="5"/>
@@ -2351,127 +2399,127 @@
       <c r="F78" s="5"/>
       <c r="G78" s="6"/>
     </row>
-    <row r="79" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D79" s="5"/>
       <c r="E79" s="5"/>
       <c r="F79" s="5"/>
       <c r="G79" s="6"/>
     </row>
-    <row r="80" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D80" s="5"/>
       <c r="E80" s="5"/>
       <c r="F80" s="5"/>
       <c r="G80" s="6"/>
     </row>
-    <row r="81" spans="4:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="4:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D81" s="5"/>
       <c r="E81" s="5"/>
       <c r="F81" s="5"/>
       <c r="G81" s="6"/>
     </row>
-    <row r="82" spans="4:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="82" spans="4:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D82" s="5"/>
       <c r="E82" s="5"/>
       <c r="F82" s="5"/>
       <c r="G82" s="6"/>
     </row>
-    <row r="83" spans="4:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="4:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D83" s="5"/>
       <c r="E83" s="5"/>
       <c r="F83" s="5"/>
       <c r="G83" s="6"/>
     </row>
-    <row r="84" spans="4:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="84" spans="4:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D84" s="5"/>
       <c r="E84" s="5"/>
       <c r="F84" s="5"/>
       <c r="G84" s="6"/>
     </row>
-    <row r="85" spans="4:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="85" spans="4:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D85" s="5"/>
       <c r="E85" s="5"/>
       <c r="F85" s="5"/>
       <c r="G85" s="6"/>
     </row>
-    <row r="86" spans="4:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="4:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D86" s="5"/>
       <c r="E86" s="5"/>
       <c r="F86" s="5"/>
       <c r="G86" s="6"/>
     </row>
-    <row r="87" spans="4:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="87" spans="4:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D87" s="5"/>
       <c r="E87" s="5"/>
       <c r="F87" s="5"/>
       <c r="G87" s="6"/>
     </row>
-    <row r="88" spans="4:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="88" spans="4:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D88" s="5"/>
       <c r="E88" s="5"/>
       <c r="F88" s="5"/>
       <c r="G88" s="6"/>
     </row>
-    <row r="89" spans="4:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="89" spans="4:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D89" s="5"/>
       <c r="E89" s="5"/>
       <c r="F89" s="5"/>
       <c r="G89" s="6"/>
     </row>
-    <row r="90" spans="4:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="90" spans="4:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D90" s="5"/>
       <c r="E90" s="5"/>
       <c r="F90" s="5"/>
       <c r="G90" s="6"/>
     </row>
-    <row r="91" spans="4:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="91" spans="4:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D91" s="5"/>
       <c r="E91" s="5"/>
       <c r="F91" s="5"/>
       <c r="G91" s="6"/>
     </row>
-    <row r="92" spans="4:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="92" spans="4:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D92" s="5"/>
       <c r="E92" s="5"/>
       <c r="F92" s="5"/>
       <c r="G92" s="6"/>
     </row>
-    <row r="93" spans="4:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="93" spans="4:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D93" s="5"/>
       <c r="E93" s="5"/>
       <c r="F93" s="5"/>
       <c r="G93" s="6"/>
     </row>
-    <row r="94" spans="4:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="94" spans="4:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D94" s="5"/>
       <c r="E94" s="5"/>
       <c r="F94" s="5"/>
       <c r="G94" s="6"/>
     </row>
-    <row r="95" spans="4:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="95" spans="4:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D95" s="5"/>
       <c r="E95" s="5"/>
       <c r="F95" s="5"/>
       <c r="G95" s="6"/>
     </row>
-    <row r="96" spans="4:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="96" spans="4:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D96" s="5"/>
       <c r="E96" s="5"/>
       <c r="F96" s="5"/>
       <c r="G96" s="6"/>
     </row>
-    <row r="97" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="97" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D97" s="5"/>
       <c r="E97" s="5"/>
       <c r="F97" s="5"/>
       <c r="G97" s="6"/>
     </row>
-    <row r="98" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="98" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D98" s="5"/>
       <c r="E98" s="5"/>
       <c r="F98" s="5"/>
       <c r="G98" s="6"/>
     </row>
-    <row r="99" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="99" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B99" s="3"/>
       <c r="C99" s="3"/>
       <c r="D99" s="11"/>
@@ -2479,7 +2527,7 @@
       <c r="F99" s="11"/>
       <c r="G99" s="12"/>
     </row>
-    <row r="100" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="100" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B100" s="3"/>
       <c r="C100" s="3"/>
       <c r="D100" s="5"/>
@@ -2487,7 +2535,7 @@
       <c r="F100" s="5"/>
       <c r="G100" s="6"/>
     </row>
-    <row r="101" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="101" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B101" s="3"/>
       <c r="C101" s="3"/>
       <c r="D101" s="5"/>
@@ -2495,19 +2543,19 @@
       <c r="F101" s="5"/>
       <c r="G101" s="6"/>
     </row>
-    <row r="102" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="102" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D102" s="5"/>
       <c r="E102" s="5"/>
       <c r="F102" s="5"/>
       <c r="G102" s="6"/>
     </row>
-    <row r="103" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="103" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D103" s="5"/>
       <c r="E103" s="5"/>
       <c r="F103" s="5"/>
       <c r="G103" s="6"/>
     </row>
-    <row r="104" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="104" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B104" s="16"/>
       <c r="C104" s="16"/>
       <c r="D104" s="5"/>
@@ -2515,7 +2563,7 @@
       <c r="F104" s="5"/>
       <c r="G104" s="6"/>
     </row>
-    <row r="105" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="105" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D105" s="5"/>
       <c r="E105" s="5"/>
       <c r="F105" s="5"/>
@@ -2535,20 +2583,20 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4DEFA5D-C6DF-4BEE-A0BF-87172BA2BD41}">
   <dimension ref="B1:G96"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="2.5703125" style="2" customWidth="1"/>
-    <col min="2" max="2" width="6.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="25.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="2.5546875" style="2" customWidth="1"/>
+    <col min="2" max="2" width="6.5546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="25.109375" style="2" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="24" style="2" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="24" style="2" customWidth="1"/>
-    <col min="6" max="6" width="30.85546875" style="2" customWidth="1"/>
-    <col min="7" max="7" width="8.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="8" max="16384" width="9.140625" style="2"/>
+    <col min="6" max="6" width="30.88671875" style="2" customWidth="1"/>
+    <col min="7" max="7" width="8.5546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="8" max="16384" width="9.109375" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:7" ht="8.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="2" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:7" ht="8.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="22" t="s">
         <v>8</v>
       </c>
@@ -2568,7 +2616,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="2:7" s="1" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:7" s="1" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B3">
         <v>1</v>
       </c>
@@ -2586,7 +2634,7 @@
       </c>
       <c r="G3" s="23"/>
     </row>
-    <row r="4" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4">
         <v>2</v>
       </c>
@@ -2604,7 +2652,7 @@
       </c>
       <c r="G4" s="23"/>
     </row>
-    <row r="5" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5">
         <v>3</v>
       </c>
@@ -2622,7 +2670,7 @@
       </c>
       <c r="G5" s="23"/>
     </row>
-    <row r="6" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6">
         <v>4</v>
       </c>
@@ -2640,7 +2688,7 @@
       </c>
       <c r="G6" s="23"/>
     </row>
-    <row r="7" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7">
         <v>5</v>
       </c>
@@ -2660,7 +2708,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B8">
         <v>6</v>
       </c>
@@ -2680,7 +2728,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9">
         <v>7</v>
       </c>
@@ -2698,7 +2746,7 @@
       </c>
       <c r="G9" s="23"/>
     </row>
-    <row r="10" spans="2:7" s="4" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:7" s="4" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10">
         <v>8</v>
       </c>
@@ -2716,7 +2764,7 @@
       </c>
       <c r="G10" s="23"/>
     </row>
-    <row r="11" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11">
         <v>9</v>
       </c>
@@ -2734,7 +2782,7 @@
       </c>
       <c r="G11" s="25"/>
     </row>
-    <row r="12" spans="2:7" s="1" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:7" s="1" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12">
         <v>10</v>
       </c>
@@ -2752,7 +2800,7 @@
       </c>
       <c r="G12" s="25"/>
     </row>
-    <row r="13" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B13" s="1"/>
       <c r="C13" s="1"/>
       <c r="D13" s="7"/>
@@ -2760,13 +2808,13 @@
       <c r="F13" s="7"/>
       <c r="G13" s="8"/>
     </row>
-    <row r="14" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D14" s="5"/>
       <c r="E14" s="5"/>
       <c r="F14" s="5"/>
       <c r="G14" s="6"/>
     </row>
-    <row r="15" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
       <c r="D15" s="5"/>
@@ -2774,7 +2822,7 @@
       <c r="F15" s="5"/>
       <c r="G15" s="6"/>
     </row>
-    <row r="16" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="3"/>
       <c r="C16" s="3"/>
       <c r="D16" s="5"/>
@@ -2782,13 +2830,13 @@
       <c r="F16" s="5"/>
       <c r="G16" s="6"/>
     </row>
-    <row r="17" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D17" s="5"/>
       <c r="E17" s="5"/>
       <c r="F17" s="5"/>
       <c r="G17" s="6"/>
     </row>
-    <row r="18" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
       <c r="D18" s="5"/>
@@ -2796,31 +2844,31 @@
       <c r="F18" s="5"/>
       <c r="G18" s="6"/>
     </row>
-    <row r="19" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D19" s="5"/>
       <c r="E19" s="5"/>
       <c r="F19" s="5"/>
       <c r="G19" s="6"/>
     </row>
-    <row r="20" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D20" s="7"/>
       <c r="E20" s="7"/>
       <c r="F20" s="7"/>
       <c r="G20" s="8"/>
     </row>
-    <row r="21" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D21" s="7"/>
       <c r="E21" s="7"/>
       <c r="F21" s="7"/>
       <c r="G21" s="8"/>
     </row>
-    <row r="22" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D22" s="5"/>
       <c r="E22" s="5"/>
       <c r="F22" s="5"/>
       <c r="G22" s="6"/>
     </row>
-    <row r="23" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B23" s="3"/>
       <c r="C23" s="3"/>
       <c r="D23" s="5"/>
@@ -2828,7 +2876,7 @@
       <c r="F23" s="5"/>
       <c r="G23" s="6"/>
     </row>
-    <row r="24" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B24" s="2"/>
       <c r="C24" s="2"/>
       <c r="D24" s="5"/>
@@ -2836,7 +2884,7 @@
       <c r="F24" s="5"/>
       <c r="G24" s="6"/>
     </row>
-    <row r="25" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B25" s="3"/>
       <c r="C25" s="3"/>
       <c r="D25" s="5"/>
@@ -2844,7 +2892,7 @@
       <c r="F25" s="5"/>
       <c r="G25" s="6"/>
     </row>
-    <row r="26" spans="2:7" s="4" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:7" s="4" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B26" s="2"/>
       <c r="C26" s="2"/>
       <c r="D26" s="5"/>
@@ -2852,37 +2900,37 @@
       <c r="F26" s="5"/>
       <c r="G26" s="6"/>
     </row>
-    <row r="27" spans="2:7" s="4" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:7" s="4" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D27" s="9"/>
       <c r="E27" s="9"/>
       <c r="F27" s="10"/>
       <c r="G27" s="9"/>
     </row>
-    <row r="28" spans="2:7" s="4" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:7" s="4" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D28" s="9"/>
       <c r="E28" s="9"/>
       <c r="F28" s="10"/>
       <c r="G28" s="9"/>
     </row>
-    <row r="29" spans="2:7" s="4" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:7" s="4" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D29" s="9"/>
       <c r="E29" s="9"/>
       <c r="F29" s="10"/>
       <c r="G29" s="9"/>
     </row>
-    <row r="30" spans="2:7" s="4" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:7" s="4" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D30" s="9"/>
       <c r="E30" s="9"/>
       <c r="F30" s="10"/>
       <c r="G30" s="9"/>
     </row>
-    <row r="31" spans="2:7" s="4" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:7" s="4" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D31" s="9"/>
       <c r="E31" s="9"/>
       <c r="F31" s="10"/>
       <c r="G31" s="9"/>
     </row>
-    <row r="32" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B32" s="4"/>
       <c r="C32" s="4"/>
       <c r="D32" s="9"/>
@@ -2890,13 +2938,13 @@
       <c r="F32" s="10"/>
       <c r="G32" s="9"/>
     </row>
-    <row r="33" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D33" s="11"/>
       <c r="E33" s="11"/>
       <c r="F33" s="11"/>
       <c r="G33" s="12"/>
     </row>
-    <row r="34" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B34" s="2"/>
       <c r="C34" s="2"/>
       <c r="D34" s="5"/>
@@ -2904,7 +2952,7 @@
       <c r="F34" s="5"/>
       <c r="G34" s="6"/>
     </row>
-    <row r="35" spans="2:7" s="13" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:7" s="13" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B35" s="3"/>
       <c r="C35" s="3"/>
       <c r="D35" s="5"/>
@@ -2912,7 +2960,7 @@
       <c r="F35" s="5"/>
       <c r="G35" s="6"/>
     </row>
-    <row r="36" spans="2:7" s="4" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:7" s="4" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B36" s="13"/>
       <c r="C36" s="13"/>
       <c r="D36" s="11"/>
@@ -2920,25 +2968,25 @@
       <c r="F36" s="11"/>
       <c r="G36" s="12"/>
     </row>
-    <row r="37" spans="2:7" s="4" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:7" s="4" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D37" s="11"/>
       <c r="E37" s="11"/>
       <c r="F37" s="11"/>
       <c r="G37" s="12"/>
     </row>
-    <row r="38" spans="2:7" s="4" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:7" s="4" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D38" s="11"/>
       <c r="E38" s="11"/>
       <c r="F38" s="11"/>
       <c r="G38" s="12"/>
     </row>
-    <row r="39" spans="2:7" s="4" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:7" s="4" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D39" s="11"/>
       <c r="E39" s="11"/>
       <c r="F39" s="11"/>
       <c r="G39" s="12"/>
     </row>
-    <row r="40" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B40" s="4"/>
       <c r="C40" s="4"/>
       <c r="D40" s="14"/>
@@ -2946,25 +2994,25 @@
       <c r="F40" s="14"/>
       <c r="G40" s="15"/>
     </row>
-    <row r="41" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D41" s="5"/>
       <c r="E41" s="5"/>
       <c r="F41" s="5"/>
       <c r="G41" s="6"/>
     </row>
-    <row r="42" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D42" s="5"/>
       <c r="E42" s="5"/>
       <c r="F42" s="5"/>
       <c r="G42" s="6"/>
     </row>
-    <row r="43" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D43" s="5"/>
       <c r="E43" s="5"/>
       <c r="F43" s="5"/>
       <c r="G43" s="6"/>
     </row>
-    <row r="44" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B44" s="2"/>
       <c r="C44" s="2"/>
       <c r="D44" s="5"/>
@@ -2972,19 +3020,19 @@
       <c r="F44" s="5"/>
       <c r="G44" s="6"/>
     </row>
-    <row r="45" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D45" s="5"/>
       <c r="E45" s="5"/>
       <c r="F45" s="5"/>
       <c r="G45" s="6"/>
     </row>
-    <row r="46" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D46" s="11"/>
       <c r="E46" s="11"/>
       <c r="F46" s="11"/>
       <c r="G46" s="12"/>
     </row>
-    <row r="47" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B47" s="3"/>
       <c r="C47" s="3"/>
       <c r="D47" s="11"/>
@@ -2992,43 +3040,43 @@
       <c r="F47" s="11"/>
       <c r="G47" s="12"/>
     </row>
-    <row r="48" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D48" s="5"/>
       <c r="E48" s="5"/>
       <c r="F48" s="5"/>
       <c r="G48" s="6"/>
     </row>
-    <row r="49" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D49" s="5"/>
       <c r="E49" s="5"/>
       <c r="F49" s="5"/>
       <c r="G49" s="6"/>
     </row>
-    <row r="50" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D50" s="11"/>
       <c r="E50" s="11"/>
       <c r="F50" s="11"/>
       <c r="G50" s="12"/>
     </row>
-    <row r="51" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D51" s="5"/>
       <c r="E51" s="5"/>
       <c r="F51" s="5"/>
       <c r="G51" s="6"/>
     </row>
-    <row r="52" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D52" s="5"/>
       <c r="E52" s="5"/>
       <c r="F52" s="5"/>
       <c r="G52" s="6"/>
     </row>
-    <row r="53" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D53" s="5"/>
       <c r="E53" s="5"/>
       <c r="F53" s="5"/>
       <c r="G53" s="6"/>
     </row>
-    <row r="54" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B54" s="2"/>
       <c r="C54" s="2"/>
       <c r="D54" s="5"/>
@@ -3036,19 +3084,19 @@
       <c r="F54" s="5"/>
       <c r="G54" s="6"/>
     </row>
-    <row r="55" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D55" s="5"/>
       <c r="E55" s="5"/>
       <c r="F55" s="5"/>
       <c r="G55" s="6"/>
     </row>
-    <row r="56" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D56" s="5"/>
       <c r="E56" s="5"/>
       <c r="F56" s="5"/>
       <c r="G56" s="6"/>
     </row>
-    <row r="57" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B57" s="3"/>
       <c r="C57" s="3"/>
       <c r="D57" s="5"/>
@@ -3056,121 +3104,121 @@
       <c r="F57" s="5"/>
       <c r="G57" s="6"/>
     </row>
-    <row r="58" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D58" s="5"/>
       <c r="E58" s="5"/>
       <c r="F58" s="5"/>
       <c r="G58" s="6"/>
     </row>
-    <row r="59" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D59" s="5"/>
       <c r="E59" s="5"/>
       <c r="F59" s="5"/>
       <c r="G59" s="6"/>
     </row>
-    <row r="60" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D60" s="5"/>
       <c r="E60" s="5"/>
       <c r="F60" s="5"/>
       <c r="G60" s="6"/>
     </row>
-    <row r="61" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D61" s="5"/>
       <c r="E61" s="5"/>
       <c r="F61" s="5"/>
       <c r="G61" s="6"/>
     </row>
-    <row r="62" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D62" s="5"/>
       <c r="E62" s="5"/>
       <c r="F62" s="5"/>
       <c r="G62" s="6"/>
     </row>
-    <row r="63" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D63" s="5"/>
       <c r="E63" s="5"/>
       <c r="F63" s="5"/>
       <c r="G63" s="6"/>
     </row>
-    <row r="64" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D64" s="5"/>
       <c r="E64" s="5"/>
       <c r="F64" s="5"/>
       <c r="G64" s="6"/>
     </row>
-    <row r="65" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D65" s="5"/>
       <c r="E65" s="5"/>
       <c r="F65" s="5"/>
       <c r="G65" s="6"/>
     </row>
-    <row r="66" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D66" s="5"/>
       <c r="E66" s="5"/>
       <c r="F66" s="5"/>
       <c r="G66" s="6"/>
     </row>
-    <row r="67" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D67" s="5"/>
       <c r="E67" s="5"/>
       <c r="F67" s="5"/>
       <c r="G67" s="6"/>
     </row>
-    <row r="68" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D68" s="5"/>
       <c r="E68" s="5"/>
       <c r="F68" s="5"/>
       <c r="G68" s="6"/>
     </row>
-    <row r="69" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D69" s="5"/>
       <c r="E69" s="5"/>
       <c r="F69" s="5"/>
       <c r="G69" s="6"/>
     </row>
-    <row r="70" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D70" s="5"/>
       <c r="E70" s="5"/>
       <c r="F70" s="5"/>
       <c r="G70" s="6"/>
     </row>
-    <row r="71" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D71" s="5"/>
       <c r="E71" s="5"/>
       <c r="F71" s="5"/>
       <c r="G71" s="6"/>
     </row>
-    <row r="72" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D72" s="5"/>
       <c r="E72" s="5"/>
       <c r="F72" s="5"/>
       <c r="G72" s="6"/>
     </row>
-    <row r="73" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D73" s="5"/>
       <c r="E73" s="5"/>
       <c r="F73" s="5"/>
       <c r="G73" s="6"/>
     </row>
-    <row r="74" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D74" s="5"/>
       <c r="E74" s="5"/>
       <c r="F74" s="5"/>
       <c r="G74" s="6"/>
     </row>
-    <row r="75" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D75" s="5"/>
       <c r="E75" s="5"/>
       <c r="F75" s="5"/>
       <c r="G75" s="6"/>
     </row>
-    <row r="76" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D76" s="5"/>
       <c r="E76" s="5"/>
       <c r="F76" s="5"/>
       <c r="G76" s="6"/>
     </row>
-    <row r="77" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B77" s="2"/>
       <c r="C77" s="2"/>
       <c r="D77" s="5"/>
@@ -3178,19 +3226,19 @@
       <c r="F77" s="5"/>
       <c r="G77" s="6"/>
     </row>
-    <row r="78" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D78" s="11"/>
       <c r="E78" s="11"/>
       <c r="F78" s="11"/>
       <c r="G78" s="12"/>
     </row>
-    <row r="79" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D79" s="5"/>
       <c r="E79" s="5"/>
       <c r="F79" s="5"/>
       <c r="G79" s="6"/>
     </row>
-    <row r="80" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B80" s="3"/>
       <c r="C80" s="3"/>
       <c r="D80" s="5"/>
@@ -3198,13 +3246,13 @@
       <c r="F80" s="5"/>
       <c r="G80" s="6"/>
     </row>
-    <row r="81" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D81" s="5"/>
       <c r="E81" s="5"/>
       <c r="F81" s="5"/>
       <c r="G81" s="6"/>
     </row>
-    <row r="82" spans="2:7" s="16" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="82" spans="2:7" s="16" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B82" s="2"/>
       <c r="C82" s="2"/>
       <c r="D82" s="5"/>
@@ -3212,7 +3260,7 @@
       <c r="F82" s="5"/>
       <c r="G82" s="6"/>
     </row>
-    <row r="83" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B83" s="16"/>
       <c r="C83" s="16"/>
       <c r="D83" s="5"/>
@@ -3220,20 +3268,20 @@
       <c r="F83" s="5"/>
       <c r="G83" s="6"/>
     </row>
-    <row r="84" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="84" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D84" s="5"/>
       <c r="E84" s="5"/>
       <c r="F84" s="5"/>
       <c r="G84" s="6"/>
     </row>
-    <row r="85" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="86" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="87" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="88" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="89" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="90" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="91" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="96" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="85" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="86" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="87" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="88" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="89" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="90" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="91" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="96" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <conditionalFormatting sqref="D3:D12">
     <cfRule type="duplicateValues" dxfId="4" priority="3"/>

</xml_diff>

<commit_message>
InstantLoan currency int to string
</commit_message>
<xml_diff>
--- a/IA_CCBS_BANK_SIDE/AccountOther/LoanAccountOpening_InstantProcess.xlsx
+++ b/IA_CCBS_BANK_SIDE/AccountOther/LoanAccountOpening_InstantProcess.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kmilos\source\repos\iApply_CCBS_API\IA_CCBS_BANK_SIDE\AccountOther\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4234C863-96FE-4972-B220-969F8E23A493}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D155E4EF-17CF-43A2-A095-CAF2649A74DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{68F28061-2ECD-4B0A-AB1D-3A449686159F}"/>
   </bookViews>
@@ -535,7 +535,7 @@
     <xf numFmtId="0" fontId="12" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="12" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -614,7 +614,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="20% - Accent4" xfId="1" builtinId="42"/>
@@ -1660,7 +1659,7 @@
         <v>24</v>
       </c>
       <c r="E11" s="26" t="s">
-        <v>4</v>
+        <v>111</v>
       </c>
       <c r="F11" s="26" t="s">
         <v>32</v>
@@ -2031,10 +2030,10 @@
       <c r="B32">
         <v>30</v>
       </c>
-      <c r="C32" s="28" t="s">
+      <c r="C32" s="26" t="s">
         <v>107</v>
       </c>
-      <c r="D32" s="28" t="s">
+      <c r="D32" s="26" t="s">
         <v>107</v>
       </c>
       <c r="E32" s="26" t="s">
@@ -2043,16 +2042,16 @@
       <c r="F32" s="26" t="s">
         <v>32</v>
       </c>
-      <c r="G32" s="28"/>
+      <c r="G32" s="26"/>
     </row>
     <row r="33" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B33">
         <v>31</v>
       </c>
-      <c r="C33" s="28" t="s">
+      <c r="C33" s="26" t="s">
         <v>108</v>
       </c>
-      <c r="D33" s="28" t="s">
+      <c r="D33" s="26" t="s">
         <v>108</v>
       </c>
       <c r="E33" s="26" t="s">
@@ -2061,25 +2060,25 @@
       <c r="F33" s="26" t="s">
         <v>32</v>
       </c>
-      <c r="G33" s="28"/>
+      <c r="G33" s="26"/>
     </row>
     <row r="34" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B34">
         <v>32</v>
       </c>
-      <c r="C34" s="28" t="s">
+      <c r="C34" s="26" t="s">
         <v>109</v>
       </c>
-      <c r="D34" s="28" t="s">
+      <c r="D34" s="26" t="s">
         <v>109</v>
       </c>
-      <c r="E34" s="28" t="s">
+      <c r="E34" s="26" t="s">
         <v>111</v>
       </c>
       <c r="F34" s="26" t="s">
         <v>32</v>
       </c>
-      <c r="G34" s="28"/>
+      <c r="G34" s="26"/>
     </row>
     <row r="35" spans="2:7" s="3" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B35" s="2"/>

</xml_diff>

<commit_message>
CreateInstantLoan request changed two fields
</commit_message>
<xml_diff>
--- a/IA_CCBS_BANK_SIDE/AccountOther/LoanAccountOpening_InstantProcess.xlsx
+++ b/IA_CCBS_BANK_SIDE/AccountOther/LoanAccountOpening_InstantProcess.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kmilos\source\repos\iApply_CCBS_API\IA_CCBS_BANK_SIDE\AccountOther\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D155E4EF-17CF-43A2-A095-CAF2649A74DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DD8362C-B59F-443D-A3BD-791538BF55DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{68F28061-2ECD-4B0A-AB1D-3A449686159F}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="113">
   <si>
     <t>Description</t>
   </si>
@@ -367,6 +367,9 @@
   </si>
   <si>
     <t>string</t>
+  </si>
+  <si>
+    <t>varchar (20)</t>
   </si>
 </sst>
 </file>
@@ -1983,7 +1986,7 @@
         <v>78</v>
       </c>
       <c r="E29" s="26" t="s">
-        <v>4</v>
+        <v>112</v>
       </c>
       <c r="F29" s="26" t="s">
         <v>32</v>
@@ -2001,7 +2004,7 @@
         <v>80</v>
       </c>
       <c r="E30" s="26" t="s">
-        <v>4</v>
+        <v>112</v>
       </c>
       <c r="F30" s="26" t="s">
         <v>32</v>

</xml_diff>